<commit_message>
10:38 time 24.07.2025 date
</commit_message>
<xml_diff>
--- a/file_service/qabul.xlsx
+++ b/file_service/qabul.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M237"/>
+  <dimension ref="A1:M256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40.42578125" customWidth="1" min="1" max="1"/>
@@ -13941,6 +13941,1089 @@
         </is>
       </c>
     </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Xusenov Anis Naufarovich</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Rus tili</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>AD3186658</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>50206066110072</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Samarqand viloyati</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>Samarqand tumani</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>998950904404</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>+998950904404</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>2025-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Quziboyev Mehriddin Jaxongirovich</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>AD8538383</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>50112075650028</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>Qashqadaryo viloyati</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>Qarshi tumani</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>998955253313</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>+998914743435</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>2025-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Solijonov obidjon axror ogli</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>AE1978187</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>50606086820106</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>Toshkent viloyati</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>Yangiyoʻl tumani</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>998994028939</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>+998953510002</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>2025-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Mingboshiyev Behro'z Dilshod o'g'li</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>AD4356766</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>51601076410036</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Sirdaryo viloyati</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>Guliston tumani</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>998944234434</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>+998944234434</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>2025-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Raimjonova Aminabonu</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>AD0405710</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>62505056730047</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>Toshkent shahri</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>Olmazor tumani</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>998935182505</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>+998935182505</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>2025-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Saidov Lazizbek Latifjon ogli</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>AD3132398</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>50304076930069</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>Toshkent shahri</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>Mirzo Ulugʻbek tumani</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>998881420703</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>+998881420703</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>2025-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Yoldoshov Ulugbek Anvarovich</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>AD8274466</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>50408085320032</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>Toshkent shahri</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>Yunusobod tumani</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>998941220359</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>+998994198080</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>2025-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Axmedova Mavsuma Yaxshiboevna</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Psixologiya</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>AD4026627</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>41807843990014</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>Samarqand viloyati</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>Urgut tumani</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>998979268084</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>+998979268084</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Asrolova Ezoza Bobir qizi</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>AD4405589</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>62108075520044</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>Jizzax viloyati</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>Forish tumani</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>998954647007</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>+998954647007</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Urakov Dilmurod</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Mehnat muhofazasi va texnika xavfsizligi</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>AD3864089</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>52806075850028</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>Navoiy viloyati</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>Zarafshon shahri</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>998931129716</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>+998931129716</t>
+        </is>
+      </c>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Sultonmurodova Sevinch Sanjarovna</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Rus tili</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>AD4231746</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>62306076840026</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>Toshkent viloyati</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>Angren shahri</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>998933233122</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>+998936683122</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Rizayeva Nigoraxon Sadikovna</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Mehnat muhofazasi va texnika xavfsizligi</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Rus tili</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>AD6008106</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>42511841230032</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>Andijon viloyati</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>Andijon shahri</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>998889941720</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>+998884222261</t>
+        </is>
+      </c>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Yusupjonova Sevinch</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Rus tili</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>AE3369465</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>61608066560040</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>Toshkent shahri</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>Sergeli tumani</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>998974235989</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>+998971432402</t>
+        </is>
+      </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Aslonova Sabrina</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>AD8337762</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>62108075790045</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>Navoiy viloyati</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>Navoiy shahri</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>998936637874</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>+998936637874</t>
+        </is>
+      </c>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Shukurullayev Adham Javlonbekovich</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>AD5041031</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>53110076100017</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>Navoiy viloyati</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>Navoiy shahri</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>998930029066</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>+998970869066</t>
+        </is>
+      </c>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Pirmahammatov Fazliddin Sherali ogli</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>AD5610246</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>50409075720119</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>Toshkent shahri</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>Mirzo Ulugʻbek tumani</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>998944135002</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>+998333003917</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Narzullayev shaxzod sherali ogli</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Hayot faoliyati xavfsizligi</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>AD8513979</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>52101086510018</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Toshkent shahri</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>Mirobod tumani</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>998337212108</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>+998337212108</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Shodiqulov shohruh shahobiddinovich</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Yurisprudensiya</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Rus tili</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>AD9483081</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>50704085800027</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>Navoiy viloyati</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>Nurota tumani</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>998507190002</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>+998507190002</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>2025-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Mirzaboyev Javoxir</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Metrologiya va standartlashtirish</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>O'zbek tili</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Kunduzgi</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>AD4390816</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>30207976690023</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>Toshkent viloyati</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>Oqqoʻrgʻon tumani</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>998975470704</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>+998975470704</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>2025-07-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="D1:D66"/>
   <mergeCells count="1">

</xml_diff>